<commit_message>
feat(schoolweek): improve school week management with enhanced validation and UI
- Add validation for school week value range (1-52)
- Improve school week combobox search functionality
- Enhance pagination component responsiveness
- Refactor import modal with better error handling and preview
- Fix formatSelect utility to use correct key for labels
- Update action cell to handle multiple school weeks
- Sort school weeks by value in container
</commit_message>
<xml_diff>
--- a/public/template_file/schoolweek-template.xlsx
+++ b/public/template_file/schoolweek-template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zena\Downloads\SMK Web\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bkt-workspace\SmartKidWeb\smartkids-tvmn\public\template_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4DBD8AE-42D0-4A9A-BA0F-B51657A4C71B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609340E0-B432-4DC8-8B98-E2FD81EC1896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6585" yWindow="6975" windowWidth="21195" windowHeight="11295" xr2:uid="{4338DCA1-FD51-4796-BBF0-1AA8D62E2AA7}"/>
+    <workbookView xWindow="5250" yWindow="1095" windowWidth="21600" windowHeight="11295" xr2:uid="{4338DCA1-FD51-4796-BBF0-1AA8D62E2AA7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D13F1CBD-E7F4-4E9C-9870-370D6F70A260}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="2"/>
@@ -421,17 +421,12 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>1</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>